<commit_message>
chore: update sample data files
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sample_data2_1.xlsx
+++ b/data/sample_data2_1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\00.디혁\01.태블로\04.개발(문서)\20260323_계리\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MALIFE\Documents\Actuarial-Report\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -437,7 +437,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="3">
-        <v>3.2428223220736498</v>
+        <v>2.7428223220736498</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -451,7 +451,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>2.9392687998764702</v>
+        <v>2.4392687998764702</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -465,7 +465,7 @@
         <v>6</v>
       </c>
       <c r="D4" s="3">
-        <v>3.1217963021535202</v>
+        <v>2.6217963021535202</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -479,7 +479,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="3">
-        <v>3.2465292532833701</v>
+        <v>2.7465292532833701</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -493,7 +493,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="3">
-        <v>2.9552897486417899</v>
+        <v>2.4552897486417899</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -507,7 +507,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="3">
-        <v>3.1304367030650799</v>
+        <v>2.6304367030650799</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -521,7 +521,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="3">
-        <v>3.2712452461088901</v>
+        <v>2.7712452461088901</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -535,7 +535,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="3">
-        <v>3.2452935959906402</v>
+        <v>2.7452935959906402</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -549,7 +549,7 @@
         <v>5</v>
       </c>
       <c r="D10" s="3">
-        <v>2.8025675768118101</v>
+        <v>2.3025675768118101</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -563,7 +563,7 @@
         <v>5</v>
       </c>
       <c r="D11" s="3">
-        <v>2.9626848035541098</v>
+        <v>2.4626848035541098</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -577,7 +577,7 @@
         <v>6</v>
       </c>
       <c r="D12" s="3">
-        <v>3.08970919385452</v>
+        <v>2.58970919385452</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -591,7 +591,7 @@
         <v>6</v>
       </c>
       <c r="D13" s="4">
-        <v>3.1329055109289698</v>
+        <v>2.6329055109289698</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -605,7 +605,7 @@
         <v>4</v>
       </c>
       <c r="D14" s="4">
-        <v>3.22799581721624</v>
+        <v>2.72799581721624</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -619,7 +619,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="4">
-        <v>2.8838293145679401</v>
+        <v>2.3838293145679401</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -633,7 +633,7 @@
         <v>6</v>
       </c>
       <c r="D16" s="4">
-        <v>3.0946450762787001</v>
+        <v>2.5946450762787001</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -647,7 +647,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="4">
-        <v>3.2341732903626901</v>
+        <v>2.7341732903626901</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -661,7 +661,7 @@
         <v>5</v>
       </c>
       <c r="D18" s="4">
-        <v>2.91339363313454</v>
+        <v>2.41339363313454</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -675,7 +675,7 @@
         <v>6</v>
       </c>
       <c r="D19" s="4">
-        <v>3.1082198699838401</v>
+        <v>2.6082198699838401</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -689,7 +689,7 @@
         <v>4</v>
       </c>
       <c r="D20" s="4">
-        <v>3.2193479240813798</v>
+        <v>2.7193479240813798</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="D21" s="4">
-        <v>2.96638251359715</v>
+        <v>2.46638251359715</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -717,7 +717,7 @@
         <v>6</v>
       </c>
       <c r="D22" s="4">
-        <v>3.1205620133374099</v>
+        <v>2.6205620133374099</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -731,7 +731,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="4">
-        <v>3.2366443745040598</v>
+        <v>2.7366443745040598</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -745,7 +745,7 @@
         <v>4</v>
       </c>
       <c r="D24" s="4">
-        <v>3.2193479240813798</v>
+        <v>2.7193479240813798</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -759,7 +759,7 @@
         <v>5</v>
       </c>
       <c r="D25" s="4">
-        <v>2.9405010994119101</v>
+        <v>2.4405010994119101</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -773,7 +773,7 @@
         <v>5</v>
       </c>
       <c r="D26" s="4">
-        <v>2.96145226058995</v>
+        <v>2.46145226058995</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -787,7 +787,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="4">
-        <v>3.1205620133374099</v>
+        <v>2.6205620133374099</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -801,7 +801,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="4">
-        <v>3.1180934763319201</v>
+        <v>2.6180934763319201</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -815,7 +815,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="4">
-        <v>3.2687734027844599</v>
+        <v>2.7687734027844599</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -829,7 +829,7 @@
         <v>5</v>
       </c>
       <c r="D30" s="4">
-        <v>2.7508861994914202</v>
+        <v>2.2508861994914202</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -843,7 +843,7 @@
         <v>6</v>
       </c>
       <c r="D31" s="4">
-        <v>3.0687341101586698</v>
+        <v>2.5687341101586698</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -857,7 +857,7 @@
         <v>4</v>
       </c>
       <c r="D32" s="4">
-        <v>3.2786611014990101</v>
+        <v>2.7786611014990101</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -871,7 +871,7 @@
         <v>5</v>
       </c>
       <c r="D33" s="4">
-        <v>2.8419598567255502</v>
+        <v>2.3419598567255502</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -885,7 +885,7 @@
         <v>6</v>
       </c>
       <c r="D34" s="4">
-        <v>3.1082198699838401</v>
+        <v>2.6082198699838401</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -899,7 +899,7 @@
         <v>4</v>
       </c>
       <c r="D35" s="4">
-        <v>3.2168772194520501</v>
+        <v>2.7168772194520501</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -913,7 +913,7 @@
         <v>5</v>
       </c>
       <c r="D36" s="4">
-        <v>2.9528248385337199</v>
+        <v>2.4528248385337199</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -927,11 +927,12 @@
         <v>6</v>
       </c>
       <c r="D37" s="4">
-        <v>3.11315656482547</v>
+        <v>2.61315656482547</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>